<commit_message>
Hold number formats to what Excel writes
The formatter's own tests used expectations written by hand. Thirty-eight
format cases now go through Excel like the rest of the parity suite, and
three of them disagreed: General keeps 0.000001 in decimal form while it
shows as many digits as scientific form would, a fraction is the last
continued-fraction convergent rather than the closest fraction (Excel
writes 1/7, not 14/99), and a negative number shown as zeros takes no
minus sign.
</commit_message>
<xml_diff>
--- a/apps/web/tests/fixtures/excel-parity.xlsx
+++ b/apps/web/tests/fixtures/excel-parity.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nico.franke/Library/Containers/com.microsoft.Excel/Data/chat-golden/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543ECB06-07B4-E44F-83B7-0CB056AC6C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6F09098-927F-4B40-A710-DBEBB3AD7BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="34560" windowHeight="22340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="481">
   <si>
     <t>operators: 1+2*3</t>
   </si>
@@ -1334,6 +1334,120 @@
   </si>
   <si>
     <t>features: WEEKNUM(DATE(2025,1,1),21)</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.00001234,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.0001234,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.000001,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1/3,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(-1/7,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(12345678901,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(123456789012,"General")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1234567,"0.0,,")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1234567,"0,")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1.25,"# ?/?")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(2.14159,"# ??/??")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.3,"# ?/8")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(2,"# ?/?")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(2.5,"?/?")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.333,"# ?/?")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(150,"[&gt;100]""big"";""small""")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(50,"[&gt;100]""big"";""small""")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(-5,"0;[Red]0")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0,"0.00;-0.00;""zero""")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1.5,"[h]:mm")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.25+1.5/86400,"hh:mm:ss.0")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.75,"h:mm a/p")</t>
+  </si>
+  <si>
+    <t>formats: TEXT("abc","0;0;0;""x""@")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1.005,"0.00")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(-0.4,"0")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(2.5,"0")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.5,"#.##")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(12.5,".00")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(123456789,"000-00-0000")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(12345,"##0.0E+0")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(0.000123,"0.00E+00")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1.5,"0.??")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(45292,"mmmmm")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(45292,"d-mmm-yy")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(45292.75,"yyyy-mm-dd hh:mm:ss")</t>
+  </si>
+  <si>
+    <t>formats: TEXT(1234.5,"#,##0.00 [$€-407]")</t>
+  </si>
+  <si>
+    <t>formats: FIXED(-1234.567,-2)</t>
+  </si>
+  <si>
+    <t>formats: DOLLAR(-0.5)</t>
   </si>
   <si>
     <t>b</t>
@@ -1416,7 +1530,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1545,39 +1659,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1586,7 +1700,7 @@
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -1629,7 +1743,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1638,7 +1752,7 @@
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -1690,168 +1804,168 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B419"/>
+  <dimension ref="A1:B457"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -5623,6 +5737,348 @@
       <c r="B419">
         <f>WEEKNUM(DATE(2025,1,1),21)</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="420" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A420" t="s">
+        <v>419</v>
+      </c>
+      <c r="B420" t="str">
+        <f>TEXT(0.00001234,"General")</f>
+        <v>0.00001234</v>
+      </c>
+    </row>
+    <row r="421" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A421" t="s">
+        <v>420</v>
+      </c>
+      <c r="B421" t="str">
+        <f>TEXT(0.0001234,"General")</f>
+        <v>0.0001234</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A422" t="s">
+        <v>421</v>
+      </c>
+      <c r="B422" t="str">
+        <f>TEXT(0.000001,"General")</f>
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A423" t="s">
+        <v>422</v>
+      </c>
+      <c r="B423" t="str">
+        <f>TEXT(1/3,"General")</f>
+        <v>0.333333333</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A424" t="s">
+        <v>423</v>
+      </c>
+      <c r="B424" t="str">
+        <f>TEXT(-1/7,"General")</f>
+        <v>-0.142857143</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A425" t="s">
+        <v>424</v>
+      </c>
+      <c r="B425" t="str">
+        <f>TEXT(12345678901,"General")</f>
+        <v>12345678901</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A426" t="s">
+        <v>425</v>
+      </c>
+      <c r="B426" t="str">
+        <f>TEXT(123456789012,"General")</f>
+        <v>1.23457E+11</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A427" t="s">
+        <v>426</v>
+      </c>
+      <c r="B427" t="str">
+        <f>TEXT(1234567,"0.0,,")</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A428" t="s">
+        <v>427</v>
+      </c>
+      <c r="B428" t="str">
+        <f>TEXT(1234567,"0,")</f>
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A429" t="s">
+        <v>428</v>
+      </c>
+      <c r="B429" t="str">
+        <f>TEXT(1.25,"# ?/?")</f>
+        <v>1 1/4</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A430" t="s">
+        <v>429</v>
+      </c>
+      <c r="B430" t="str">
+        <f>TEXT(2.14159,"# ??/??")</f>
+        <v xml:space="preserve">2  1/7 </v>
+      </c>
+    </row>
+    <row r="431" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A431" t="s">
+        <v>430</v>
+      </c>
+      <c r="B431" t="str">
+        <f>TEXT(0.3,"# ?/8")</f>
+        <v xml:space="preserve"> 2/8</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A432" t="s">
+        <v>431</v>
+      </c>
+      <c r="B432" t="str">
+        <f>TEXT(2,"# ?/?")</f>
+        <v xml:space="preserve">2    </v>
+      </c>
+    </row>
+    <row r="433" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A433" t="s">
+        <v>432</v>
+      </c>
+      <c r="B433" t="str">
+        <f>TEXT(2.5,"?/?")</f>
+        <v>5/2</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A434" t="s">
+        <v>433</v>
+      </c>
+      <c r="B434" t="str">
+        <f>TEXT(0.333,"# ?/?")</f>
+        <v xml:space="preserve"> 1/3</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A435" t="s">
+        <v>434</v>
+      </c>
+      <c r="B435" t="str">
+        <f>TEXT(150,"[&gt;100]""big"";""small""")</f>
+        <v>big</v>
+      </c>
+    </row>
+    <row r="436" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A436" t="s">
+        <v>435</v>
+      </c>
+      <c r="B436" t="str">
+        <f>TEXT(50,"[&gt;100]""big"";""small""")</f>
+        <v>small</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A437" t="s">
+        <v>436</v>
+      </c>
+      <c r="B437" t="str">
+        <f>TEXT(-5,"0;[Red]0")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A438" t="s">
+        <v>437</v>
+      </c>
+      <c r="B438" t="str">
+        <f>TEXT(0,"0.00;-0.00;""zero""")</f>
+        <v>zero</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A439" t="s">
+        <v>438</v>
+      </c>
+      <c r="B439" t="str">
+        <f>TEXT(1.5,"[h]:mm")</f>
+        <v>36:00</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A440" t="s">
+        <v>439</v>
+      </c>
+      <c r="B440" t="str">
+        <f>TEXT(0.25+1.5/86400,"hh:mm:ss.0")</f>
+        <v>06:00:01.5</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A441" t="s">
+        <v>440</v>
+      </c>
+      <c r="B441" t="str">
+        <f>TEXT(0.75,"h:mm a/p")</f>
+        <v>6:00 p</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A442" t="s">
+        <v>441</v>
+      </c>
+      <c r="B442" t="str">
+        <f>TEXT("abc","0;0;0;""x""@")</f>
+        <v>xabc</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A443" t="s">
+        <v>442</v>
+      </c>
+      <c r="B443" t="str">
+        <f>TEXT(1.005,"0.00")</f>
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A444" t="s">
+        <v>443</v>
+      </c>
+      <c r="B444" t="str">
+        <f>TEXT(-0.4,"0")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A445" t="s">
+        <v>444</v>
+      </c>
+      <c r="B445" t="str">
+        <f>TEXT(2.5,"0")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A446" t="s">
+        <v>445</v>
+      </c>
+      <c r="B446" t="str">
+        <f>TEXT(0.5,"#.##")</f>
+        <v>.5</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A447" t="s">
+        <v>446</v>
+      </c>
+      <c r="B447" t="str">
+        <f>TEXT(12.5,".00")</f>
+        <v>12.50</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A448" t="s">
+        <v>447</v>
+      </c>
+      <c r="B448" t="str">
+        <f>TEXT(123456789,"000-00-0000")</f>
+        <v>123-45-6789</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A449" t="s">
+        <v>448</v>
+      </c>
+      <c r="B449" t="str">
+        <f>TEXT(12345,"##0.0E+0")</f>
+        <v>12.3E+3</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A450" t="s">
+        <v>449</v>
+      </c>
+      <c r="B450" t="str">
+        <f>TEXT(0.000123,"0.00E+00")</f>
+        <v>1.23E-04</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A451" t="s">
+        <v>450</v>
+      </c>
+      <c r="B451" t="str">
+        <f>TEXT(1.5,"0.??")</f>
+        <v xml:space="preserve">1.5 </v>
+      </c>
+    </row>
+    <row r="452" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A452" t="s">
+        <v>451</v>
+      </c>
+      <c r="B452" t="str">
+        <f>TEXT(45292,"mmmmm")</f>
+        <v>J</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A453" t="s">
+        <v>452</v>
+      </c>
+      <c r="B453" t="str">
+        <f>TEXT(45292,"d-mmm-yy")</f>
+        <v>1-Jan-24</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A454" t="s">
+        <v>453</v>
+      </c>
+      <c r="B454" t="str">
+        <f>TEXT(45292.75,"yyyy-mm-dd hh:mm:ss")</f>
+        <v>2024-01-01 18:00:00</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A455" t="s">
+        <v>454</v>
+      </c>
+      <c r="B455" t="str">
+        <f>TEXT(1234.5,"#,##0.00 [$€-407]")</f>
+        <v>1,234.50 €</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A456" t="s">
+        <v>455</v>
+      </c>
+      <c r="B456" t="str">
+        <f>FIXED(-1234.567,-2)</f>
+        <v>-1,200</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A457" t="s">
+        <v>456</v>
+      </c>
+      <c r="B457" t="str">
+        <f>DOLLAR(-0.5)</f>
+        <v>($0.50)</v>
       </c>
     </row>
   </sheetData>
@@ -5632,7 +6088,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E5017"/>
+  <dimension ref="A1:E5473"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -9937,6 +10393,348 @@
       <c r="B5017">
         <f>WEEKNUM(DATE(2025,1,1),21)</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="5029" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5029" t="s">
+        <v>419</v>
+      </c>
+      <c r="B5029" t="str">
+        <f>TEXT(0.00001234,"General")</f>
+        <v>0.00001234</v>
+      </c>
+    </row>
+    <row r="5041" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5041" t="s">
+        <v>420</v>
+      </c>
+      <c r="B5041" t="str">
+        <f>TEXT(0.0001234,"General")</f>
+        <v>0.0001234</v>
+      </c>
+    </row>
+    <row r="5053" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5053" t="s">
+        <v>421</v>
+      </c>
+      <c r="B5053" t="str">
+        <f>TEXT(0.000001,"General")</f>
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row r="5065" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5065" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5065" t="str">
+        <f>TEXT(1/3,"General")</f>
+        <v>0.333333333</v>
+      </c>
+    </row>
+    <row r="5077" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5077" t="s">
+        <v>423</v>
+      </c>
+      <c r="B5077" t="str">
+        <f>TEXT(-1/7,"General")</f>
+        <v>-0.142857143</v>
+      </c>
+    </row>
+    <row r="5089" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5089" t="s">
+        <v>424</v>
+      </c>
+      <c r="B5089" t="str">
+        <f>TEXT(12345678901,"General")</f>
+        <v>12345678901</v>
+      </c>
+    </row>
+    <row r="5101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5101" t="s">
+        <v>425</v>
+      </c>
+      <c r="B5101" t="str">
+        <f>TEXT(123456789012,"General")</f>
+        <v>1.23457E+11</v>
+      </c>
+    </row>
+    <row r="5113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5113" t="s">
+        <v>426</v>
+      </c>
+      <c r="B5113" t="str">
+        <f>TEXT(1234567,"0.0,,")</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="5125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5125" t="s">
+        <v>427</v>
+      </c>
+      <c r="B5125" t="str">
+        <f>TEXT(1234567,"0,")</f>
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="5137" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5137" t="s">
+        <v>428</v>
+      </c>
+      <c r="B5137" t="str">
+        <f>TEXT(1.25,"# ?/?")</f>
+        <v>1 1/4</v>
+      </c>
+    </row>
+    <row r="5149" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5149" t="s">
+        <v>429</v>
+      </c>
+      <c r="B5149" t="str">
+        <f>TEXT(2.14159,"# ??/??")</f>
+        <v xml:space="preserve">2  1/7 </v>
+      </c>
+    </row>
+    <row r="5161" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5161" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5161" t="str">
+        <f>TEXT(0.3,"# ?/8")</f>
+        <v xml:space="preserve"> 2/8</v>
+      </c>
+    </row>
+    <row r="5173" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5173" t="s">
+        <v>431</v>
+      </c>
+      <c r="B5173" t="str">
+        <f>TEXT(2,"# ?/?")</f>
+        <v xml:space="preserve">2    </v>
+      </c>
+    </row>
+    <row r="5185" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5185" t="s">
+        <v>432</v>
+      </c>
+      <c r="B5185" t="str">
+        <f>TEXT(2.5,"?/?")</f>
+        <v>5/2</v>
+      </c>
+    </row>
+    <row r="5197" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5197" t="s">
+        <v>433</v>
+      </c>
+      <c r="B5197" t="str">
+        <f>TEXT(0.333,"# ?/?")</f>
+        <v xml:space="preserve"> 1/3</v>
+      </c>
+    </row>
+    <row r="5209" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5209" t="s">
+        <v>434</v>
+      </c>
+      <c r="B5209" t="str">
+        <f>TEXT(150,"[&gt;100]""big"";""small""")</f>
+        <v>big</v>
+      </c>
+    </row>
+    <row r="5221" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5221" t="s">
+        <v>435</v>
+      </c>
+      <c r="B5221" t="str">
+        <f>TEXT(50,"[&gt;100]""big"";""small""")</f>
+        <v>small</v>
+      </c>
+    </row>
+    <row r="5233" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5233" t="s">
+        <v>436</v>
+      </c>
+      <c r="B5233" t="str">
+        <f>TEXT(-5,"0;[Red]0")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5245" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5245" t="s">
+        <v>437</v>
+      </c>
+      <c r="B5245" t="str">
+        <f>TEXT(0,"0.00;-0.00;""zero""")</f>
+        <v>zero</v>
+      </c>
+    </row>
+    <row r="5257" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5257" t="s">
+        <v>438</v>
+      </c>
+      <c r="B5257" t="str">
+        <f>TEXT(1.5,"[h]:mm")</f>
+        <v>36:00</v>
+      </c>
+    </row>
+    <row r="5269" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5269" t="s">
+        <v>439</v>
+      </c>
+      <c r="B5269" t="str">
+        <f>TEXT(0.25+1.5/86400,"hh:mm:ss.0")</f>
+        <v>06:00:01.5</v>
+      </c>
+    </row>
+    <row r="5281" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5281" t="s">
+        <v>440</v>
+      </c>
+      <c r="B5281" t="str">
+        <f>TEXT(0.75,"h:mm a/p")</f>
+        <v>6:00 p</v>
+      </c>
+    </row>
+    <row r="5293" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5293" t="s">
+        <v>441</v>
+      </c>
+      <c r="B5293" t="str">
+        <f>TEXT("abc","0;0;0;""x""@")</f>
+        <v>xabc</v>
+      </c>
+    </row>
+    <row r="5305" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5305" t="s">
+        <v>442</v>
+      </c>
+      <c r="B5305" t="str">
+        <f>TEXT(1.005,"0.00")</f>
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="5317" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5317" t="s">
+        <v>443</v>
+      </c>
+      <c r="B5317" t="str">
+        <f>TEXT(-0.4,"0")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5329" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5329" t="s">
+        <v>444</v>
+      </c>
+      <c r="B5329" t="str">
+        <f>TEXT(2.5,"0")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5341" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5341" t="s">
+        <v>445</v>
+      </c>
+      <c r="B5341" t="str">
+        <f>TEXT(0.5,"#.##")</f>
+        <v>.5</v>
+      </c>
+    </row>
+    <row r="5353" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5353" t="s">
+        <v>446</v>
+      </c>
+      <c r="B5353" t="str">
+        <f>TEXT(12.5,".00")</f>
+        <v>12.50</v>
+      </c>
+    </row>
+    <row r="5365" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5365" t="s">
+        <v>447</v>
+      </c>
+      <c r="B5365" t="str">
+        <f>TEXT(123456789,"000-00-0000")</f>
+        <v>123-45-6789</v>
+      </c>
+    </row>
+    <row r="5377" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5377" t="s">
+        <v>448</v>
+      </c>
+      <c r="B5377" t="str">
+        <f>TEXT(12345,"##0.0E+0")</f>
+        <v>12.3E+3</v>
+      </c>
+    </row>
+    <row r="5389" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5389" t="s">
+        <v>449</v>
+      </c>
+      <c r="B5389" t="str">
+        <f>TEXT(0.000123,"0.00E+00")</f>
+        <v>1.23E-04</v>
+      </c>
+    </row>
+    <row r="5401" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5401" t="s">
+        <v>450</v>
+      </c>
+      <c r="B5401" t="str">
+        <f>TEXT(1.5,"0.??")</f>
+        <v xml:space="preserve">1.5 </v>
+      </c>
+    </row>
+    <row r="5413" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5413" t="s">
+        <v>451</v>
+      </c>
+      <c r="B5413" t="str">
+        <f>TEXT(45292,"mmmmm")</f>
+        <v>J</v>
+      </c>
+    </row>
+    <row r="5425" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5425" t="s">
+        <v>452</v>
+      </c>
+      <c r="B5425" t="str">
+        <f>TEXT(45292,"d-mmm-yy")</f>
+        <v>1-Jan-24</v>
+      </c>
+    </row>
+    <row r="5437" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5437" t="s">
+        <v>453</v>
+      </c>
+      <c r="B5437" t="str">
+        <f>TEXT(45292.75,"yyyy-mm-dd hh:mm:ss")</f>
+        <v>2024-01-01 18:00:00</v>
+      </c>
+    </row>
+    <row r="5449" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5449" t="s">
+        <v>454</v>
+      </c>
+      <c r="B5449" t="str">
+        <f>TEXT(1234.5,"#,##0.00 [$€-407]")</f>
+        <v>1,234.50 €</v>
+      </c>
+    </row>
+    <row r="5461" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5461" t="s">
+        <v>455</v>
+      </c>
+      <c r="B5461" t="str">
+        <f>FIXED(-1234.567,-2)</f>
+        <v>-1,200</v>
+      </c>
+    </row>
+    <row r="5473" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5473" t="s">
+        <v>456</v>
+      </c>
+      <c r="B5473" t="str">
+        <f>DOLLAR(-0.5)</f>
+        <v>($0.50)</v>
       </c>
     </row>
   </sheetData>
@@ -9951,28 +10749,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>433</v>
+        <v>471</v>
       </c>
       <c r="B1" t="s">
-        <v>434</v>
+        <v>472</v>
       </c>
       <c r="C1" t="s">
-        <v>435</v>
+        <v>473</v>
       </c>
       <c r="D1" t="s">
-        <v>436</v>
+        <v>474</v>
       </c>
       <c r="E1" t="s">
-        <v>437</v>
+        <v>475</v>
       </c>
       <c r="F1" t="s">
-        <v>438</v>
+        <v>476</v>
       </c>
       <c r="G1" t="s">
-        <v>439</v>
+        <v>477</v>
       </c>
       <c r="H1" t="s">
-        <v>440</v>
+        <v>478</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -9980,7 +10778,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>431</v>
+        <v>469</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -9989,7 +10787,7 @@
         <v>45292</v>
       </c>
       <c r="E2" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="F2">
         <v>10</v>
@@ -10006,16 +10804,16 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>429</v>
+        <v>467</v>
       </c>
       <c r="C3" t="s">
-        <v>430</v>
+        <v>468</v>
       </c>
       <c r="D3">
         <v>45329</v>
       </c>
       <c r="E3" t="s">
-        <v>419</v>
+        <v>457</v>
       </c>
       <c r="F3">
         <v>20</v>
@@ -10032,7 +10830,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>428</v>
+        <v>466</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -10041,7 +10839,7 @@
         <v>45366</v>
       </c>
       <c r="E4" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="F4">
         <v>30</v>
@@ -10058,13 +10856,13 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>427</v>
+        <v>465</v>
       </c>
       <c r="D5">
         <v>45403</v>
       </c>
       <c r="E5" t="s">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="F5">
         <v>40</v>
@@ -10081,7 +10879,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>426</v>
+        <v>464</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -10090,7 +10888,7 @@
         <v>45440</v>
       </c>
       <c r="E6" t="s">
-        <v>419</v>
+        <v>457</v>
       </c>
       <c r="F6">
         <v>50</v>
@@ -10107,16 +10905,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>424</v>
+        <v>462</v>
       </c>
       <c r="C7" t="s">
-        <v>425</v>
+        <v>463</v>
       </c>
       <c r="D7">
         <v>45477</v>
       </c>
       <c r="E7" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="F7">
         <v>60</v>
@@ -10133,7 +10931,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -10142,7 +10940,7 @@
         <v>45514</v>
       </c>
       <c r="E8" t="s">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="F8">
         <v>70</v>
@@ -10159,7 +10957,7 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>422</v>
+        <v>460</v>
       </c>
       <c r="C9" t="b">
         <v>0</v>
@@ -10168,7 +10966,7 @@
         <v>45551</v>
       </c>
       <c r="E9" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="F9">
         <v>80</v>
@@ -10185,7 +10983,7 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>421</v>
+        <v>459</v>
       </c>
       <c r="C10">
         <v>-2</v>
@@ -10194,7 +10992,7 @@
         <v>45588</v>
       </c>
       <c r="E10" t="s">
-        <v>419</v>
+        <v>457</v>
       </c>
       <c r="F10">
         <v>90</v>
@@ -10211,7 +11009,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>432</v>
+        <v>470</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -10220,7 +11018,7 @@
         <v>45625</v>
       </c>
       <c r="E11" t="s">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="F11">
         <v>100</v>
@@ -10250,7 +11048,7 @@
         <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>442</v>
+        <v>480</v>
       </c>
       <c r="D1" t="str">
         <f>TEXT(1234.5,"#,##0.00")</f>

</xml_diff>